<commit_message>
update prompt.html iterative tuning, renderer labels, scores csv/xlsx, run scripts
</commit_message>
<xml_diff>
--- a/src/scores_all.xlsx
+++ b/src/scores_all.xlsx
@@ -33428,22 +33428,22 @@
         </is>
       </c>
       <c r="F524" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G524" t="n">
         <v>3</v>
       </c>
       <c r="H524" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I524" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J524" t="n">
         <v>3</v>
       </c>
       <c r="K524" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L524" t="b">
         <v>0</v>
@@ -33620,19 +33620,19 @@
         <v>4</v>
       </c>
       <c r="G527" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H527" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I527" t="n">
         <v>4</v>
       </c>
       <c r="J527" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K527" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L527" t="b">
         <v>0</v>
@@ -33680,22 +33680,22 @@
         </is>
       </c>
       <c r="F528" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G528" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H528" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I528" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J528" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K528" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="L528" t="b">
         <v>0</v>
@@ -34754,19 +34754,19 @@
         <v>4</v>
       </c>
       <c r="G545" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H545" t="n">
         <v>4</v>
       </c>
       <c r="I545" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J545" t="n">
         <v>4</v>
       </c>
       <c r="K545" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L545" t="b">
         <v>0</v>
@@ -34943,19 +34943,19 @@
         <v>4</v>
       </c>
       <c r="G548" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H548" t="n">
         <v>4</v>
       </c>
       <c r="I548" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J548" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K548" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L548" t="b">
         <v>0</v>
@@ -35015,10 +35015,10 @@
         <v>4</v>
       </c>
       <c r="J549" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K549" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L549" t="b">
         <v>0</v>
@@ -35138,13 +35138,13 @@
         <v>4</v>
       </c>
       <c r="I551" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J551" t="n">
         <v>3</v>
       </c>
       <c r="K551" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L551" t="b">
         <v>0</v>
@@ -36464,10 +36464,10 @@
         <v>4</v>
       </c>
       <c r="J572" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K572" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L572" t="b">
         <v>0</v>
@@ -36527,10 +36527,10 @@
         <v>4</v>
       </c>
       <c r="J573" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K573" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L573" t="b">
         <v>0</v>
@@ -36647,16 +36647,16 @@
         <v>4</v>
       </c>
       <c r="H575" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I575" t="n">
         <v>4</v>
       </c>
       <c r="J575" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K575" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L575" t="b">
         <v>0</v>
@@ -36716,10 +36716,10 @@
         <v>4</v>
       </c>
       <c r="J576" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K576" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L576" t="b">
         <v>0</v>
@@ -37787,10 +37787,10 @@
         <v>4</v>
       </c>
       <c r="J593" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K593" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L593" t="b">
         <v>0</v>
@@ -37970,10 +37970,10 @@
         <v>3</v>
       </c>
       <c r="H596" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I596" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J596" t="n">
         <v>3</v>
@@ -38039,10 +38039,10 @@
         <v>4</v>
       </c>
       <c r="J597" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K597" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L597" t="b">
         <v>0</v>
@@ -38165,10 +38165,10 @@
         <v>4</v>
       </c>
       <c r="J599" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K599" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L599" t="b">
         <v>0</v>
@@ -38216,7 +38216,7 @@
         </is>
       </c>
       <c r="F600" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G600" t="n">
         <v>4</v>
@@ -38231,7 +38231,7 @@
         <v>3</v>
       </c>
       <c r="K600" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L600" t="b">
         <v>0</v>
@@ -39290,7 +39290,7 @@
         <v>4</v>
       </c>
       <c r="G617" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H617" t="n">
         <v>4</v>
@@ -39302,7 +39302,7 @@
         <v>4</v>
       </c>
       <c r="K617" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L617" t="b">
         <v>0</v>
@@ -39479,19 +39479,19 @@
         <v>4</v>
       </c>
       <c r="G620" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H620" t="n">
         <v>4</v>
       </c>
       <c r="I620" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J620" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K620" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L620" t="b">
         <v>0</v>
@@ -39551,10 +39551,10 @@
         <v>4</v>
       </c>
       <c r="J621" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K621" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L621" t="b">
         <v>0</v>
@@ -39668,19 +39668,19 @@
         <v>4</v>
       </c>
       <c r="G623" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H623" t="n">
         <v>4</v>
       </c>
       <c r="I623" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J623" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K623" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L623" t="b">
         <v>0</v>
@@ -39728,22 +39728,22 @@
         </is>
       </c>
       <c r="F624" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G624" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H624" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I624" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J624" t="n">
         <v>3</v>
       </c>
       <c r="K624" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L624" t="b">
         <v>0</v>
@@ -40613,19 +40613,19 @@
         <v>4</v>
       </c>
       <c r="G638" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H638" t="n">
         <v>4</v>
       </c>
       <c r="I638" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J638" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K638" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L638" t="b">
         <v>0</v>
@@ -40802,13 +40802,13 @@
         <v>4</v>
       </c>
       <c r="G641" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H641" t="n">
         <v>4</v>
       </c>
       <c r="I641" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J641" t="n">
         <v>4</v>
@@ -41054,7 +41054,7 @@
         <v>4</v>
       </c>
       <c r="G645" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H645" t="n">
         <v>4</v>
@@ -41063,7 +41063,7 @@
         <v>4</v>
       </c>
       <c r="J645" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K645" t="n">
         <v>19</v>
@@ -41186,13 +41186,13 @@
         <v>4</v>
       </c>
       <c r="I647" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J647" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K647" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="L647" t="b">
         <v>0</v>
@@ -42323,10 +42323,10 @@
         <v>4</v>
       </c>
       <c r="J665" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K665" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L665" t="b">
         <v>0</v>
@@ -42503,7 +42503,7 @@
         <v>4</v>
       </c>
       <c r="G668" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H668" t="n">
         <v>4</v>
@@ -42515,7 +42515,7 @@
         <v>3</v>
       </c>
       <c r="K668" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L668" t="b">
         <v>0</v>
@@ -42575,10 +42575,10 @@
         <v>4</v>
       </c>
       <c r="J669" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K669" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L669" t="b">
         <v>0</v>
@@ -42701,10 +42701,10 @@
         <v>4</v>
       </c>
       <c r="J671" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K671" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L671" t="b">
         <v>0</v>
@@ -43637,7 +43637,7 @@
         <v>4</v>
       </c>
       <c r="G686" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H686" t="n">
         <v>4</v>
@@ -43649,7 +43649,7 @@
         <v>4</v>
       </c>
       <c r="K686" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L686" t="b">
         <v>0</v>
@@ -43826,7 +43826,7 @@
         <v>4</v>
       </c>
       <c r="G689" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H689" t="n">
         <v>4</v>
@@ -43835,10 +43835,10 @@
         <v>4</v>
       </c>
       <c r="J689" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K689" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L689" t="b">
         <v>0</v>
@@ -44024,10 +44024,10 @@
         <v>4</v>
       </c>
       <c r="J692" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K692" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L692" t="b">
         <v>0</v>
@@ -44087,10 +44087,10 @@
         <v>4</v>
       </c>
       <c r="J693" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K693" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L693" t="b">
         <v>0</v>
@@ -44213,10 +44213,10 @@
         <v>4</v>
       </c>
       <c r="J695" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K695" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L695" t="b">
         <v>0</v>
@@ -44273,13 +44273,13 @@
         <v>4</v>
       </c>
       <c r="I696" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J696" t="n">
         <v>4</v>
       </c>
       <c r="K696" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L696" t="b">
         <v>0</v>
@@ -45338,19 +45338,19 @@
         <v>4</v>
       </c>
       <c r="G713" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H713" t="n">
         <v>4</v>
       </c>
       <c r="I713" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J713" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K713" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L713" t="b">
         <v>0</v>
@@ -45530,13 +45530,13 @@
         <v>3</v>
       </c>
       <c r="H716" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I716" t="n">
         <v>4</v>
       </c>
       <c r="J716" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K716" t="n">
         <v>18</v>
@@ -45599,10 +45599,10 @@
         <v>4</v>
       </c>
       <c r="J717" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K717" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L717" t="b">
         <v>0</v>
@@ -45716,19 +45716,19 @@
         <v>4</v>
       </c>
       <c r="G719" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H719" t="n">
         <v>4</v>
       </c>
       <c r="I719" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J719" t="n">
         <v>4</v>
       </c>
       <c r="K719" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L719" t="b">
         <v>0</v>
@@ -45788,10 +45788,10 @@
         <v>4</v>
       </c>
       <c r="J720" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K720" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L720" t="b">
         <v>0</v>
@@ -46664,7 +46664,7 @@
         <v>4</v>
       </c>
       <c r="H734" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I734" t="n">
         <v>4</v>
@@ -46673,7 +46673,7 @@
         <v>4</v>
       </c>
       <c r="K734" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L734" t="b">
         <v>0</v>
@@ -46850,7 +46850,7 @@
         <v>4</v>
       </c>
       <c r="G737" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H737" t="n">
         <v>4</v>
@@ -46859,7 +46859,7 @@
         <v>4</v>
       </c>
       <c r="J737" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K737" t="n">
         <v>19</v>
@@ -47231,16 +47231,16 @@
         <v>4</v>
       </c>
       <c r="H743" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I743" t="n">
         <v>4</v>
       </c>
       <c r="J743" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K743" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L743" t="b">
         <v>0</v>
@@ -47297,13 +47297,13 @@
         <v>4</v>
       </c>
       <c r="I744" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J744" t="n">
         <v>4</v>
       </c>
       <c r="K744" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L744" t="b">
         <v>0</v>
@@ -48179,13 +48179,13 @@
         <v>4</v>
       </c>
       <c r="I758" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J758" t="n">
         <v>4</v>
       </c>
       <c r="K758" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L758" t="b">
         <v>0</v>
@@ -48362,13 +48362,13 @@
         <v>4</v>
       </c>
       <c r="G761" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H761" t="n">
         <v>4</v>
       </c>
       <c r="I761" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J761" t="n">
         <v>4</v>
@@ -48557,13 +48557,13 @@
         <v>4</v>
       </c>
       <c r="I764" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J764" t="n">
         <v>3</v>
       </c>
       <c r="K764" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L764" t="b">
         <v>0</v>
@@ -48617,7 +48617,7 @@
         <v>4</v>
       </c>
       <c r="H765" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I765" t="n">
         <v>4</v>
@@ -48626,7 +48626,7 @@
         <v>4</v>
       </c>
       <c r="K765" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L765" t="b">
         <v>0</v>
@@ -48746,13 +48746,13 @@
         <v>4</v>
       </c>
       <c r="I767" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J767" t="n">
         <v>4</v>
       </c>
       <c r="K767" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L767" t="b">
         <v>0</v>
@@ -48812,10 +48812,10 @@
         <v>4</v>
       </c>
       <c r="J768" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K768" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L768" t="b">
         <v>0</v>
@@ -49748,7 +49748,7 @@
         <v>4</v>
       </c>
       <c r="G783" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H783" t="n">
         <v>4</v>
@@ -49760,7 +49760,7 @@
         <v>4</v>
       </c>
       <c r="K783" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L783" t="b">
         <v>0</v>
@@ -49937,19 +49937,19 @@
         <v>4</v>
       </c>
       <c r="G786" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H786" t="n">
         <v>4</v>
       </c>
       <c r="I786" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J786" t="n">
         <v>3</v>
       </c>
       <c r="K786" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="L786" t="b">
         <v>0</v>
@@ -50003,16 +50003,16 @@
         <v>3</v>
       </c>
       <c r="H787" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I787" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J787" t="n">
         <v>3</v>
       </c>
       <c r="K787" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L787" t="b">
         <v>0</v>
@@ -50129,16 +50129,16 @@
         <v>4</v>
       </c>
       <c r="H789" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I789" t="n">
         <v>4</v>
       </c>
       <c r="J789" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K789" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L789" t="b">
         <v>0</v>
@@ -51260,19 +51260,19 @@
         <v>4</v>
       </c>
       <c r="G807" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H807" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I807" t="n">
         <v>4</v>
       </c>
       <c r="J807" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K807" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L807" t="b">
         <v>0</v>
@@ -51455,13 +51455,13 @@
         <v>4</v>
       </c>
       <c r="I810" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J810" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K810" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="L810" t="b">
         <v>0</v>
@@ -51512,19 +51512,19 @@
         <v>4</v>
       </c>
       <c r="G811" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H811" t="n">
         <v>4</v>
       </c>
       <c r="I811" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J811" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K811" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L811" t="b">
         <v>0</v>
@@ -52583,7 +52583,7 @@
         <v>4</v>
       </c>
       <c r="G828" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H828" t="n">
         <v>4</v>
@@ -52595,7 +52595,7 @@
         <v>4</v>
       </c>
       <c r="K828" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L828" t="b">
         <v>0</v>
@@ -52970,10 +52970,10 @@
         <v>4</v>
       </c>
       <c r="J834" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K834" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L834" t="b">
         <v>0</v>
@@ -54284,7 +54284,7 @@
         <v>4</v>
       </c>
       <c r="G855" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H855" t="n">
         <v>4</v>
@@ -54296,7 +54296,7 @@
         <v>4</v>
       </c>
       <c r="K855" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L855" t="b">
         <v>0</v>
@@ -54473,10 +54473,10 @@
         <v>4</v>
       </c>
       <c r="G858" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H858" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I858" t="n">
         <v>4</v>
@@ -54485,7 +54485,7 @@
         <v>4</v>
       </c>
       <c r="K858" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L858" t="b">
         <v>0</v>
@@ -54536,19 +54536,19 @@
         <v>4</v>
       </c>
       <c r="G859" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H859" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I859" t="n">
         <v>4</v>
       </c>
       <c r="J859" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K859" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L859" t="b">
         <v>0</v>
@@ -54662,7 +54662,7 @@
         <v>4</v>
       </c>
       <c r="G861" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H861" t="n">
         <v>4</v>
@@ -54671,10 +54671,10 @@
         <v>4</v>
       </c>
       <c r="J861" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K861" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L861" t="b">
         <v>0</v>
@@ -55796,7 +55796,7 @@
         <v>4</v>
       </c>
       <c r="G879" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H879" t="n">
         <v>4</v>
@@ -55808,7 +55808,7 @@
         <v>3</v>
       </c>
       <c r="K879" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L879" t="b">
         <v>0</v>
@@ -55985,13 +55985,13 @@
         <v>4</v>
       </c>
       <c r="G882" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H882" t="n">
         <v>4</v>
       </c>
       <c r="I882" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J882" t="n">
         <v>3</v>
@@ -56174,7 +56174,7 @@
         <v>4</v>
       </c>
       <c r="G885" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H885" t="n">
         <v>4</v>
@@ -56183,10 +56183,10 @@
         <v>4</v>
       </c>
       <c r="J885" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K885" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L885" t="b">
         <v>0</v>
@@ -57314,13 +57314,13 @@
         <v>4</v>
       </c>
       <c r="I903" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J903" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K903" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L903" t="b">
         <v>0</v>
@@ -57497,7 +57497,7 @@
         <v>4</v>
       </c>
       <c r="G906" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H906" t="n">
         <v>4</v>
@@ -57506,10 +57506,10 @@
         <v>4</v>
       </c>
       <c r="J906" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K906" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L906" t="b">
         <v>0</v>
@@ -57560,7 +57560,7 @@
         <v>4</v>
       </c>
       <c r="G907" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H907" t="n">
         <v>4</v>
@@ -57572,7 +57572,7 @@
         <v>3</v>
       </c>
       <c r="K907" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L907" t="b">
         <v>0</v>
@@ -57758,10 +57758,10 @@
         <v>4</v>
       </c>
       <c r="J910" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K910" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L910" t="b">
         <v>0</v>
@@ -58823,16 +58823,16 @@
         <v>4</v>
       </c>
       <c r="H927" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I927" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J927" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K927" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L927" t="b">
         <v>0</v>
@@ -58892,13 +58892,13 @@
         <v>4</v>
       </c>
       <c r="J928" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K928" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L928" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M928" t="b">
         <v>0</v>
@@ -58913,7 +58913,7 @@
         <v>0</v>
       </c>
       <c r="Q928" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="929">
@@ -58952,13 +58952,13 @@
         <v>4</v>
       </c>
       <c r="I929" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J929" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K929" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L929" t="b">
         <v>0</v>
@@ -59012,7 +59012,7 @@
         <v>3</v>
       </c>
       <c r="H930" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I930" t="n">
         <v>4</v>
@@ -59021,7 +59021,7 @@
         <v>3</v>
       </c>
       <c r="K930" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L930" t="b">
         <v>0</v>
@@ -59072,19 +59072,19 @@
         <v>4</v>
       </c>
       <c r="G931" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H931" t="n">
         <v>4</v>
       </c>
       <c r="I931" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J931" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K931" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L931" t="b">
         <v>0</v>
@@ -59204,10 +59204,10 @@
         <v>4</v>
       </c>
       <c r="I933" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J933" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K933" t="n">
         <v>19</v>

</xml_diff>